<commit_message>
Adiciona fundos de capa e integra aos sete editores
</commit_message>
<xml_diff>
--- a/conteudo/topo-de-funil/planejamento-carrosseis.xlsx
+++ b/conteudo/topo-de-funil/planejamento-carrosseis.xlsx
@@ -549,7 +549,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Roteiro pronto; imagens pendentes</t>
+          <t>Roteiro e fundo da capa prontos; revisar composição e exportar</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Roteiro pronto; imagens pendentes</t>
+          <t>Roteiro e fundo da capa prontos; revisar composição e exportar</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Roteiro pronto; imagens pendentes</t>
+          <t>Roteiro e fundo da capa prontos; revisar composição e exportar</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Roteiro pronto; imagens pendentes</t>
+          <t>Roteiro e fundo da capa prontos; revisar composição e exportar</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Roteiro pronto; imagens pendentes</t>
+          <t>Roteiro e fundo da capa prontos; revisar composição e exportar</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Roteiro pronto; imagens pendentes</t>
+          <t>Roteiro e fundo da capa prontos; revisar composição e exportar</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Roteiro pronto; imagens pendentes</t>
+          <t>Roteiro e fundo da capa prontos; revisar composição e exportar</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -5396,12 +5396,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>84 prompts prontos; geração não executada</t>
+          <t>7 fundos de capa gerados e inseridos; imagens internas e stories não gerados.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finaliza 56 slides e 28 stories com pacotes e indice de publicacao
</commit_message>
<xml_diff>
--- a/conteudo/topo-de-funil/planejamento-carrosseis.xlsx
+++ b/conteudo/topo-de-funil/planejamento-carrosseis.xlsx
@@ -549,7 +549,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Roteiro e fundo da capa prontos; revisar composição e exportar</t>
+          <t>PNG exportado e conferido; não publicado</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Roteiro e fundo da capa prontos; revisar composição e exportar</t>
+          <t>PNG exportado e conferido; não publicado</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Roteiro e fundo da capa prontos; revisar composição e exportar</t>
+          <t>PNG exportado e conferido; não publicado</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Roteiro e fundo da capa prontos; revisar composição e exportar</t>
+          <t>PNG exportado e conferido; não publicado</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Roteiro e fundo da capa prontos; revisar composição e exportar</t>
+          <t>PNG exportado e conferido; não publicado</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Roteiro e fundo da capa prontos; revisar composição e exportar</t>
+          <t>PNG exportado e conferido; não publicado</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Roteiro e fundo da capa prontos; revisar composição e exportar</t>
+          <t>PNG exportado e conferido; não publicado</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -5396,12 +5396,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Parcial</t>
+          <t>Concluído para esta série</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>7 fundos de capa gerados e inseridos; imagens internas e stories não gerados.</t>
+          <t>7 capas com IA; internos tipográficos; 56 slides e 28 stories exportados. Prompts alternativos preservados.</t>
         </is>
       </c>
     </row>

</xml_diff>